<commit_message>
Add new concept image and update peri-urban opportunity Excel file
- Introduced a new image file, `concept_improved.jpeg`, to enhance visual representation of project concepts.
- Updated the `opportunities_periurban_fchip_2026-07.xlsx` file to reflect the latest data changes, ensuring accurate and relevant information for funding opportunities.
</commit_message>
<xml_diff>
--- a/opportunities/opportunities_periurban_fchip_2026-07.xlsx
+++ b/opportunities/opportunities_periurban_fchip_2026-07.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding\apps\flutter\fairbanks\opportunities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F28373F8-4004-44DA-9723-AC1BFA3C9285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59CAA001-6976-4BCE-AE3D-C5592B363701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -300,7 +300,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,8 +334,48 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -369,6 +409,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -397,7 +449,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -432,6 +484,27 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -874,130 +947,130 @@
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
     </row>
-    <row r="6" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:9" s="16" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+    </row>
+    <row r="7" spans="1:9" s="19" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+    </row>
+    <row r="8" spans="1:9" s="13" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" spans="1:9" s="22" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-    </row>
-    <row r="10" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+    </row>
+    <row r="10" spans="1:9" s="13" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
     </row>
     <row r="11" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">

</xml_diff>

<commit_message>
Update opportunities Excel files to reflect latest data changes
- Revised the `opportunities_periurban_fchip_2026-07.xlsx` and `opportunities.xlsx` files to incorporate the most recent data updates, ensuring accuracy and relevance for funding opportunities.
</commit_message>
<xml_diff>
--- a/opportunities/opportunities_periurban_fchip_2026-07.xlsx
+++ b/opportunities/opportunities_periurban_fchip_2026-07.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding\apps\flutter\fairbanks\opportunities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59CAA001-6976-4BCE-AE3D-C5592B363701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D9C4571-7EF2-4A49-80C9-F3B635EE21C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -300,7 +300,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -374,6 +374,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -446,23 +454,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -505,8 +505,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -847,308 +851,311 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="10" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:9" s="7" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-    </row>
-    <row r="3" spans="1:9" s="10" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="8" t="s">
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+    </row>
+    <row r="3" spans="1:9" s="7" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-    </row>
-    <row r="4" spans="1:9" s="13" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+    </row>
+    <row r="4" spans="1:9" s="10" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-    </row>
-    <row r="5" spans="1:9" s="13" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+    </row>
+    <row r="5" spans="1:9" s="10" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-    </row>
-    <row r="6" spans="1:9" s="16" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="14" t="s">
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+    </row>
+    <row r="6" spans="1:9" s="13" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-    </row>
-    <row r="7" spans="1:9" s="19" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="17" t="s">
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" spans="1:9" s="16" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="17" t="s">
+      <c r="G7" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-    </row>
-    <row r="8" spans="1:9" s="13" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+    </row>
+    <row r="8" spans="1:9" s="10" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-    </row>
-    <row r="9" spans="1:9" s="22" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="20" t="s">
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+    </row>
+    <row r="9" spans="1:9" s="19" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B9" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="20" t="s">
+      <c r="C9" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="21" t="s">
+      <c r="E9" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F9" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="20" t="s">
+      <c r="G9" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
-    </row>
-    <row r="10" spans="1:9" s="13" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+    </row>
+    <row r="10" spans="1:9" s="10" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-    </row>
-    <row r="11" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+    </row>
+    <row r="11" spans="1:9" s="16" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+    </row>
+    <row r="12" spans="1:9" s="10" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:9" ht="100" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" spans="1:9" s="10" customFormat="1" ht="100" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I13" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <hyperlinks>
+    <hyperlink ref="B13" r:id="rId1" xr:uid="{9C57C5E2-16E2-46FB-B367-B60907A2E3B2}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1163,122 +1170,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="4" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="4" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="4" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="4" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="4" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="4" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="4" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="56" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="4" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>